<commit_message>
Sync planning SharePoint : S45
</commit_message>
<xml_diff>
--- a/Plannings 2026 S45 v2.xlsx
+++ b/Plannings 2026 S45 v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cdalpes.sharepoint.com/sites/msteams_bd0f90/Documents partages/02. USP - TOS - General/RH/Plannings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CC0C0633-600D-4321-8C9D-1C0350CE0995}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="8_{CC0C0633-600D-4321-8C9D-1C0350CE0995}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1413E22F-501F-4485-9E25-FDDBF0CA1CF7}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="127">
   <si>
     <t>Planning des salariés du 02/11/2026 au 08/11/2026</t>
   </si>
@@ -319,9 +319,6 @@
   </si>
   <si>
     <t>RABII Mehdi</t>
-  </si>
-  <si>
-    <t>13:30/19:30</t>
   </si>
   <si>
     <t>SANGARNE Enzo</t>
@@ -924,13 +921,7 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -945,7 +936,13 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4768,21 +4765,21 @@
     <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>62</xdr:row>
+      <xdr:row>80</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>62</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="14" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7258B331-A969-426F-8840-7D671740E7BD}"/>
+      <xdr:row>80</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C8F5D026-6204-4603-9C81-20DA5483A222}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4798,7 +4795,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="18043071" y="775607"/>
+          <a:off x="18043071" y="12055929"/>
           <a:ext cx="123825" cy="123825"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -4812,21 +4809,21 @@
     <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>64</xdr:row>
+      <xdr:row>82</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>123825</xdr:colOff>
-      <xdr:row>64</xdr:row>
-      <xdr:rowOff>123825</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="79" name="Picture 1" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D6EBCB71-7027-4CD9-8FBD-BCA3A31D5798}"/>
+      <xdr:row>82</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 1" descr="Picture">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3448369A-8EAB-4B98-BA98-05F02A1921AF}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4842,7 +4839,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="18043071" y="1156607"/>
+          <a:off x="18043071" y="12436929"/>
           <a:ext cx="123825" cy="123825"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -5231,45 +5228,45 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B1" s="55" t="s">
+      <c r="B1" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="55" t="s">
+      <c r="B2" s="48" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="55"/>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
+      <c r="E2" s="48"/>
+      <c r="F2" s="48"/>
+      <c r="G2" s="48"/>
+      <c r="H2" s="48"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B3" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="C3" s="13" t="s">
         <v>124</v>
       </c>
-      <c r="C3" s="13" t="s">
+      <c r="D3" s="13" t="s">
         <v>125</v>
       </c>
-      <c r="D3" s="13" t="s">
-        <v>126</v>
-      </c>
       <c r="E3" s="13" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H3" s="13" t="s">
         <v>13</v>
@@ -5302,7 +5299,7 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="51" t="s">
+      <c r="A5" s="49" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="14"/>
@@ -5320,7 +5317,7 @@
       <c r="H5" s="16"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="52"/>
+      <c r="A6" s="50"/>
       <c r="B6" s="1"/>
       <c r="C6" s="2" t="s">
         <v>14</v>
@@ -5336,7 +5333,7 @@
       <c r="H6" s="17"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="52"/>
+      <c r="A7" s="50"/>
       <c r="B7" s="1"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
@@ -5346,7 +5343,7 @@
       <c r="H7" s="17"/>
     </row>
     <row r="8" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="53"/>
+      <c r="A8" s="51"/>
       <c r="B8" s="18"/>
       <c r="C8" s="19"/>
       <c r="D8" s="19"/>
@@ -5356,7 +5353,7 @@
       <c r="H8" s="20"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="51" t="s">
+      <c r="A9" s="49" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="15"/>
@@ -5372,7 +5369,7 @@
       <c r="H9" s="16"/>
     </row>
     <row r="10" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="53"/>
+      <c r="A10" s="51"/>
       <c r="B10" s="19"/>
       <c r="C10" s="19"/>
       <c r="D10" s="36" t="s">
@@ -5386,7 +5383,7 @@
       <c r="H10" s="20"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="51" t="s">
+      <c r="A11" s="49" t="s">
         <v>22</v>
       </c>
       <c r="B11" s="15"/>
@@ -5404,7 +5401,7 @@
       <c r="H11" s="16"/>
     </row>
     <row r="12" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="53"/>
+      <c r="A12" s="51"/>
       <c r="B12" s="19"/>
       <c r="C12" s="19" t="s">
         <v>23</v>
@@ -5423,16 +5420,16 @@
       <c r="A13" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="48"/>
-      <c r="C13" s="49"/>
-      <c r="D13" s="49"/>
-      <c r="E13" s="49"/>
-      <c r="F13" s="49"/>
-      <c r="G13" s="49"/>
-      <c r="H13" s="50"/>
+      <c r="B13" s="53"/>
+      <c r="C13" s="54"/>
+      <c r="D13" s="54"/>
+      <c r="E13" s="54"/>
+      <c r="F13" s="54"/>
+      <c r="G13" s="54"/>
+      <c r="H13" s="55"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="51" t="s">
+      <c r="A14" s="49" t="s">
         <v>26</v>
       </c>
       <c r="B14" s="15" t="s">
@@ -5442,19 +5439,19 @@
         <v>12</v>
       </c>
       <c r="D14" s="34" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E14" s="15" t="s">
         <v>12</v>
       </c>
       <c r="F14" s="15"/>
       <c r="G14" s="34" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H14" s="16"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="52"/>
+      <c r="A15" s="50"/>
       <c r="B15" s="2" t="s">
         <v>27</v>
       </c>
@@ -5462,7 +5459,7 @@
         <v>15</v>
       </c>
       <c r="D15" s="35" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>29</v>
@@ -5474,7 +5471,7 @@
       <c r="H15" s="17"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="52"/>
+      <c r="A16" s="50"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="35"/>
@@ -5486,7 +5483,7 @@
       <c r="H16" s="17"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" s="52"/>
+      <c r="A17" s="50"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="35"/>
@@ -5498,19 +5495,19 @@
       <c r="H17" s="17"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="52"/>
+      <c r="A18" s="50"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="35"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
       <c r="G18" s="32" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H18" s="17"/>
     </row>
     <row r="19" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="53"/>
+      <c r="A19" s="51"/>
       <c r="B19" s="19"/>
       <c r="C19" s="19"/>
       <c r="D19" s="36"/>
@@ -5522,7 +5519,7 @@
       <c r="H19" s="20"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="51" t="s">
+      <c r="A20" s="49" t="s">
         <v>33</v>
       </c>
       <c r="B20" s="15" t="s">
@@ -5540,7 +5537,7 @@
       <c r="H20" s="16"/>
     </row>
     <row r="21" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="53"/>
+      <c r="A21" s="51"/>
       <c r="B21" s="19" t="s">
         <v>15</v>
       </c>
@@ -5556,7 +5553,7 @@
       <c r="H21" s="20"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="51" t="s">
+      <c r="A22" s="49" t="s">
         <v>35</v>
       </c>
       <c r="B22" s="45" t="s">
@@ -5578,7 +5575,7 @@
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="52"/>
+      <c r="A23" s="50"/>
       <c r="B23" s="46" t="s">
         <v>37</v>
       </c>
@@ -5598,7 +5595,7 @@
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" s="52"/>
+      <c r="A24" s="50"/>
       <c r="B24" s="3" t="s">
         <v>12</v>
       </c>
@@ -5616,7 +5613,7 @@
       <c r="H24" s="17"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="52"/>
+      <c r="A25" s="50"/>
       <c r="B25" s="2" t="s">
         <v>42</v>
       </c>
@@ -5634,7 +5631,7 @@
       <c r="H25" s="17"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="52"/>
+      <c r="A26" s="50"/>
       <c r="B26" s="42" t="s">
         <v>45</v>
       </c>
@@ -5652,7 +5649,7 @@
       <c r="H26" s="17"/>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="52"/>
+      <c r="A27" s="50"/>
       <c r="B27" s="43" t="s">
         <v>46</v>
       </c>
@@ -5670,7 +5667,7 @@
       <c r="H27" s="17"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="52"/>
+      <c r="A28" s="50"/>
       <c r="B28" s="43"/>
       <c r="C28" s="37" t="s">
         <v>36</v>
@@ -5682,7 +5679,7 @@
       <c r="H28" s="17"/>
     </row>
     <row r="29" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="53"/>
+      <c r="A29" s="51"/>
       <c r="B29" s="44"/>
       <c r="C29" s="36" t="s">
         <v>49</v>
@@ -5694,7 +5691,7 @@
       <c r="H29" s="20"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="51" t="s">
+      <c r="A30" s="49" t="s">
         <v>50</v>
       </c>
       <c r="B30" s="15"/>
@@ -5708,7 +5705,7 @@
       <c r="H30" s="16"/>
     </row>
     <row r="31" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="53"/>
+      <c r="A31" s="51"/>
       <c r="B31" s="19"/>
       <c r="C31" s="19"/>
       <c r="D31" s="19"/>
@@ -5720,7 +5717,7 @@
       <c r="H31" s="20"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="51" t="s">
+      <c r="A32" s="49" t="s">
         <v>51</v>
       </c>
       <c r="B32" s="34" t="s">
@@ -5742,7 +5739,7 @@
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" s="52"/>
+      <c r="A33" s="50"/>
       <c r="B33" s="35" t="s">
         <v>52</v>
       </c>
@@ -5762,7 +5759,7 @@
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="52"/>
+      <c r="A34" s="50"/>
       <c r="B34" s="38" t="s">
         <v>56</v>
       </c>
@@ -5782,7 +5779,7 @@
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="52"/>
+      <c r="A35" s="50"/>
       <c r="B35" s="41" t="s">
         <v>59</v>
       </c>
@@ -5802,7 +5799,7 @@
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="52"/>
+      <c r="A36" s="50"/>
       <c r="B36" s="41"/>
       <c r="C36" s="2"/>
       <c r="D36" s="37" t="s">
@@ -5818,7 +5815,7 @@
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" s="52"/>
+      <c r="A37" s="50"/>
       <c r="B37" s="41"/>
       <c r="C37" s="2"/>
       <c r="D37" s="35" t="s">
@@ -5834,7 +5831,7 @@
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="52"/>
+      <c r="A38" s="50"/>
       <c r="B38" s="41"/>
       <c r="C38" s="2"/>
       <c r="D38" s="37" t="s">
@@ -5846,7 +5843,7 @@
       <c r="H38" s="17"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A39" s="52"/>
+      <c r="A39" s="50"/>
       <c r="B39" s="41"/>
       <c r="C39" s="2"/>
       <c r="D39" s="35" t="s">
@@ -5858,7 +5855,7 @@
       <c r="H39" s="17"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A40" s="52"/>
+      <c r="A40" s="50"/>
       <c r="B40" s="41"/>
       <c r="C40" s="2"/>
       <c r="D40" s="37" t="s">
@@ -5870,7 +5867,7 @@
       <c r="H40" s="17"/>
     </row>
     <row r="41" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="53"/>
+      <c r="A41" s="51"/>
       <c r="B41" s="39"/>
       <c r="C41" s="19"/>
       <c r="D41" s="36" t="s">
@@ -5885,16 +5882,16 @@
       <c r="A42" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="B42" s="48"/>
-      <c r="C42" s="49"/>
-      <c r="D42" s="49"/>
-      <c r="E42" s="49"/>
-      <c r="F42" s="49"/>
-      <c r="G42" s="49"/>
-      <c r="H42" s="50"/>
+      <c r="B42" s="53"/>
+      <c r="C42" s="54"/>
+      <c r="D42" s="54"/>
+      <c r="E42" s="54"/>
+      <c r="F42" s="54"/>
+      <c r="G42" s="54"/>
+      <c r="H42" s="55"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A43" s="51" t="s">
+      <c r="A43" s="49" t="s">
         <v>68</v>
       </c>
       <c r="B43" s="34" t="s">
@@ -5914,7 +5911,7 @@
       <c r="H43" s="16"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44" s="52"/>
+      <c r="A44" s="50"/>
       <c r="B44" s="35" t="s">
         <v>69</v>
       </c>
@@ -5932,7 +5929,7 @@
       <c r="H44" s="17"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A45" s="52"/>
+      <c r="A45" s="50"/>
       <c r="B45" s="35"/>
       <c r="C45" s="2"/>
       <c r="D45" s="47" t="s">
@@ -5948,7 +5945,7 @@
       <c r="H45" s="17"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A46" s="52"/>
+      <c r="A46" s="50"/>
       <c r="B46" s="35"/>
       <c r="C46" s="2"/>
       <c r="D46" s="46" t="s">
@@ -5964,7 +5961,7 @@
       <c r="H46" s="17"/>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A47" s="52"/>
+      <c r="A47" s="50"/>
       <c r="B47" s="35"/>
       <c r="C47" s="2"/>
       <c r="D47" s="37" t="s">
@@ -5976,7 +5973,7 @@
       <c r="H47" s="17"/>
     </row>
     <row r="48" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="53"/>
+      <c r="A48" s="51"/>
       <c r="B48" s="36"/>
       <c r="C48" s="19"/>
       <c r="D48" s="36" t="s">
@@ -5988,7 +5985,7 @@
       <c r="H48" s="20"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A49" s="51" t="s">
+      <c r="A49" s="49" t="s">
         <v>77</v>
       </c>
       <c r="B49" s="15"/>
@@ -6004,7 +6001,7 @@
       <c r="H49" s="16"/>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A50" s="52"/>
+      <c r="A50" s="50"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
       <c r="D50" s="35" t="s">
@@ -6018,7 +6015,7 @@
       <c r="H50" s="17"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A51" s="52"/>
+      <c r="A51" s="50"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
       <c r="D51" s="35"/>
@@ -6030,7 +6027,7 @@
       <c r="H51" s="17"/>
     </row>
     <row r="52" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="53"/>
+      <c r="A52" s="51"/>
       <c r="B52" s="19"/>
       <c r="C52" s="19"/>
       <c r="D52" s="36"/>
@@ -6042,7 +6039,7 @@
       <c r="H52" s="20"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A53" s="51" t="s">
+      <c r="A53" s="49" t="s">
         <v>78</v>
       </c>
       <c r="B53" s="15"/>
@@ -6058,7 +6055,7 @@
       <c r="H53" s="16"/>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A54" s="52"/>
+      <c r="A54" s="50"/>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
       <c r="D54" s="35" t="s">
@@ -6072,7 +6069,7 @@
       <c r="H54" s="17"/>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A55" s="52"/>
+      <c r="A55" s="50"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
       <c r="D55" s="35"/>
@@ -6084,7 +6081,7 @@
       <c r="H55" s="17"/>
     </row>
     <row r="56" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="53"/>
+      <c r="A56" s="51"/>
       <c r="B56" s="19"/>
       <c r="C56" s="19"/>
       <c r="D56" s="36"/>
@@ -6099,28 +6096,28 @@
       <c r="A57" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="B57" s="48"/>
-      <c r="C57" s="49"/>
-      <c r="D57" s="49"/>
-      <c r="E57" s="49"/>
-      <c r="F57" s="49"/>
-      <c r="G57" s="49"/>
-      <c r="H57" s="50"/>
+      <c r="B57" s="53"/>
+      <c r="C57" s="54"/>
+      <c r="D57" s="54"/>
+      <c r="E57" s="54"/>
+      <c r="F57" s="54"/>
+      <c r="G57" s="54"/>
+      <c r="H57" s="55"/>
     </row>
     <row r="58" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="B58" s="48"/>
-      <c r="C58" s="49"/>
-      <c r="D58" s="49"/>
-      <c r="E58" s="49"/>
-      <c r="F58" s="49"/>
-      <c r="G58" s="49"/>
-      <c r="H58" s="50"/>
+      <c r="B58" s="53"/>
+      <c r="C58" s="54"/>
+      <c r="D58" s="54"/>
+      <c r="E58" s="54"/>
+      <c r="F58" s="54"/>
+      <c r="G58" s="54"/>
+      <c r="H58" s="55"/>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A59" s="51" t="s">
+      <c r="A59" s="49" t="s">
         <v>81</v>
       </c>
       <c r="B59" s="15"/>
@@ -6134,7 +6131,7 @@
       <c r="H59" s="16"/>
     </row>
     <row r="60" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="53"/>
+      <c r="A60" s="51"/>
       <c r="B60" s="19"/>
       <c r="C60" s="19"/>
       <c r="D60" s="19"/>
@@ -6146,7 +6143,7 @@
       <c r="H60" s="20"/>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A61" s="51" t="s">
+      <c r="A61" s="49" t="s">
         <v>82</v>
       </c>
       <c r="B61" s="40" t="s">
@@ -6162,7 +6159,7 @@
       <c r="H61" s="16"/>
     </row>
     <row r="62" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="53"/>
+      <c r="A62" s="51"/>
       <c r="B62" s="39" t="s">
         <v>59</v>
       </c>
@@ -6176,7 +6173,7 @@
       <c r="H62" s="20"/>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A63" s="51" t="s">
+      <c r="A63" s="49" t="s">
         <v>83</v>
       </c>
       <c r="B63" s="15"/>
@@ -6184,57 +6181,49 @@
       <c r="D63" s="15"/>
       <c r="E63" s="15"/>
       <c r="F63" s="15"/>
-      <c r="G63" s="26" t="s">
-        <v>13</v>
-      </c>
+      <c r="G63" s="15"/>
       <c r="H63" s="28" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A64" s="52"/>
+      <c r="A64" s="50"/>
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
       <c r="D64" s="2"/>
       <c r="E64" s="2"/>
       <c r="F64" s="2"/>
-      <c r="G64" s="27" t="s">
-        <v>16</v>
-      </c>
+      <c r="G64" s="2"/>
       <c r="H64" s="31" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A65" s="52"/>
+      <c r="A65" s="50"/>
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
       <c r="D65" s="2"/>
       <c r="E65" s="2"/>
       <c r="F65" s="2"/>
-      <c r="G65" s="3" t="s">
-        <v>12</v>
-      </c>
+      <c r="G65" s="2"/>
       <c r="H65" s="22" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A66" s="52"/>
+      <c r="A66" s="50"/>
       <c r="B66" s="2"/>
       <c r="C66" s="2"/>
       <c r="D66" s="2"/>
       <c r="E66" s="2"/>
       <c r="F66" s="2"/>
-      <c r="G66" s="2" t="s">
-        <v>127</v>
-      </c>
+      <c r="G66" s="2"/>
       <c r="H66" s="17" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A67" s="52"/>
+      <c r="A67" s="50"/>
       <c r="B67" s="2"/>
       <c r="C67" s="2"/>
       <c r="D67" s="2"/>
@@ -6246,7 +6235,7 @@
       </c>
     </row>
     <row r="68" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="53"/>
+      <c r="A68" s="51"/>
       <c r="B68" s="19"/>
       <c r="C68" s="19"/>
       <c r="D68" s="19"/>
@@ -6258,7 +6247,7 @@
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A69" s="51" t="s">
+      <c r="A69" s="49" t="s">
         <v>86</v>
       </c>
       <c r="B69" s="15"/>
@@ -6272,7 +6261,7 @@
       <c r="H69" s="16"/>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A70" s="52"/>
+      <c r="A70" s="50"/>
       <c r="B70" s="2"/>
       <c r="C70" s="35" t="s">
         <v>52</v>
@@ -6284,7 +6273,7 @@
       <c r="H70" s="17"/>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A71" s="52"/>
+      <c r="A71" s="50"/>
       <c r="B71" s="2"/>
       <c r="C71" s="38" t="s">
         <v>56</v>
@@ -6296,7 +6285,7 @@
       <c r="H71" s="17"/>
     </row>
     <row r="72" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="53"/>
+      <c r="A72" s="51"/>
       <c r="B72" s="19"/>
       <c r="C72" s="39" t="s">
         <v>59</v>
@@ -6308,7 +6297,7 @@
       <c r="H72" s="20"/>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A73" s="51" t="s">
+      <c r="A73" s="49" t="s">
         <v>87</v>
       </c>
       <c r="B73" s="15"/>
@@ -6324,7 +6313,7 @@
       </c>
     </row>
     <row r="74" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="53"/>
+      <c r="A74" s="51"/>
       <c r="B74" s="19"/>
       <c r="C74" s="19"/>
       <c r="D74" s="19"/>
@@ -6338,7 +6327,7 @@
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A75" s="51" t="s">
+      <c r="A75" s="49" t="s">
         <v>88</v>
       </c>
       <c r="B75" s="15" t="s">
@@ -6362,7 +6351,7 @@
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A76" s="52"/>
+      <c r="A76" s="50"/>
       <c r="B76" s="2" t="s">
         <v>91</v>
       </c>
@@ -6384,7 +6373,7 @@
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A77" s="52"/>
+      <c r="A77" s="50"/>
       <c r="B77" s="23" t="s">
         <v>89</v>
       </c>
@@ -6400,13 +6389,13 @@
       <c r="H77" s="17"/>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A78" s="52"/>
+      <c r="A78" s="50"/>
       <c r="B78" s="24" t="s">
         <v>95</v>
       </c>
       <c r="C78" s="2"/>
       <c r="D78" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E78" s="2"/>
       <c r="F78" s="2"/>
@@ -6416,7 +6405,7 @@
       <c r="H78" s="17"/>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A79" s="52"/>
+      <c r="A79" s="50"/>
       <c r="B79" s="3" t="s">
         <v>12</v>
       </c>
@@ -6428,7 +6417,7 @@
       <c r="H79" s="17"/>
     </row>
     <row r="80" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="53"/>
+      <c r="A80" s="51"/>
       <c r="B80" s="19" t="s">
         <v>97</v>
       </c>
@@ -6440,7 +6429,7 @@
       <c r="H80" s="20"/>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A81" s="51" t="s">
+      <c r="A81" s="49" t="s">
         <v>98</v>
       </c>
       <c r="B81" s="15"/>
@@ -6454,19 +6443,19 @@
       <c r="H81" s="16"/>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A82" s="52"/>
+      <c r="A82" s="50"/>
       <c r="B82" s="2"/>
       <c r="C82" s="2"/>
       <c r="D82" s="2"/>
       <c r="E82" s="2"/>
       <c r="F82" s="2"/>
       <c r="G82" s="27" t="s">
-        <v>99</v>
+        <v>16</v>
       </c>
       <c r="H82" s="17"/>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A83" s="52"/>
+      <c r="A83" s="50"/>
       <c r="B83" s="2"/>
       <c r="C83" s="2"/>
       <c r="D83" s="2"/>
@@ -6478,66 +6467,66 @@
       <c r="H83" s="17"/>
     </row>
     <row r="84" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="53"/>
+      <c r="A84" s="51"/>
       <c r="B84" s="19"/>
       <c r="C84" s="19"/>
       <c r="D84" s="19"/>
       <c r="E84" s="19"/>
       <c r="F84" s="19"/>
-      <c r="G84" s="19" t="s">
-        <v>59</v>
+      <c r="G84" s="2" t="s">
+        <v>126</v>
       </c>
       <c r="H84" s="20"/>
     </row>
     <row r="85" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A85" s="21" t="s">
-        <v>100</v>
-      </c>
-      <c r="B85" s="48"/>
-      <c r="C85" s="49"/>
-      <c r="D85" s="49"/>
-      <c r="E85" s="49"/>
-      <c r="F85" s="49"/>
-      <c r="G85" s="49"/>
-      <c r="H85" s="50"/>
+        <v>99</v>
+      </c>
+      <c r="B85" s="53"/>
+      <c r="C85" s="54"/>
+      <c r="D85" s="54"/>
+      <c r="E85" s="54"/>
+      <c r="F85" s="54"/>
+      <c r="G85" s="54"/>
+      <c r="H85" s="55"/>
     </row>
     <row r="86" spans="1:8" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B86" s="54"/>
-      <c r="C86" s="54"/>
-      <c r="D86" s="54"/>
-      <c r="E86" s="54"/>
-      <c r="F86" s="54"/>
-      <c r="G86" s="54"/>
-      <c r="H86" s="54"/>
+      <c r="B86" s="52"/>
+      <c r="C86" s="52"/>
+      <c r="D86" s="52"/>
+      <c r="E86" s="52"/>
+      <c r="F86" s="52"/>
+      <c r="G86" s="52"/>
+      <c r="H86" s="52"/>
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="A5:A8"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A14:A19"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="A22:A29"/>
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="A49:A52"/>
-    <mergeCell ref="A53:A56"/>
-    <mergeCell ref="A59:A60"/>
-    <mergeCell ref="A30:A31"/>
-    <mergeCell ref="A32:A41"/>
-    <mergeCell ref="A43:A48"/>
-    <mergeCell ref="A81:A84"/>
+    <mergeCell ref="B58:H58"/>
+    <mergeCell ref="B57:H57"/>
+    <mergeCell ref="B85:H85"/>
     <mergeCell ref="B86:H86"/>
     <mergeCell ref="A61:A62"/>
     <mergeCell ref="A63:A68"/>
     <mergeCell ref="A69:A72"/>
     <mergeCell ref="A73:A74"/>
     <mergeCell ref="A75:A80"/>
+    <mergeCell ref="A59:A60"/>
+    <mergeCell ref="A30:A31"/>
+    <mergeCell ref="A32:A41"/>
+    <mergeCell ref="A43:A48"/>
+    <mergeCell ref="A81:A84"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="A22:A29"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="A49:A52"/>
+    <mergeCell ref="A53:A56"/>
     <mergeCell ref="B13:H13"/>
     <mergeCell ref="B42:H42"/>
-    <mergeCell ref="B58:H58"/>
-    <mergeCell ref="B57:H57"/>
-    <mergeCell ref="B85:H85"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="A5:A8"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A14:A19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="36" fitToHeight="0" orientation="landscape" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
@@ -6557,7 +6546,7 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B4" s="56" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C4" s="56"/>
       <c r="D4" s="56"/>
@@ -6565,7 +6554,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B5" s="57" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C5" s="57"/>
       <c r="D5" s="57"/>
@@ -6576,16 +6565,16 @@
         <v>3</v>
       </c>
       <c r="B6" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="C6" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="D6" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="E6" s="7" t="s">
         <v>107</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -6998,7 +6987,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B31" s="8">
         <v>0</v>
@@ -7015,7 +7004,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B32" s="8">
         <v>0</v>
@@ -7032,7 +7021,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B33" s="8">
         <v>0</v>
@@ -7082,21 +7071,21 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="B4" s="12" t="s">
         <v>109</v>
-      </c>
-      <c r="B4" s="12" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B5" s="12"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B6" s="12" t="s">
         <v>88</v>
@@ -7104,18 +7093,18 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="B7" s="12" t="s">
         <v>113</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="B8" s="12" t="s">
         <v>115</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -7296,13 +7285,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2758D9DD-7814-41F6-BF86-0EA16AD5C099}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38E08E73-868B-4DD9-A8E9-EB4A0151F4BC}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62965CD4-3520-439E-9283-1A81D95CB023}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{98BDD875-18A9-4A27-9982-B600AB1900E8}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2FA19422-B216-4E0D-95D9-DD1DD88788CE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D63C381-C968-4095-8EFF-D3E2059C9376}"/>
 </file>
</xml_diff>